<commit_message>
feat(estructuras): actualizar base de datos a 40 estructuras QFDOS (036-040) y v3.6.0
</commit_message>
<xml_diff>
--- a/docs/estructuras/estructuras_qfdos.xlsx
+++ b/docs/estructuras/estructuras_qfdos.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estructuras" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propiedades'!$A$1:$AF$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propiedades'!$A$1:$AF$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1017,6 +1017,131 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2381250" cy="1905000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId36"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2381250" cy="1905000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId37"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2381250" cy="1905000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId38"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2381250" cy="1905000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId39"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>40</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2381250" cy="1905000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId40"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -1309,7 +1434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF36"/>
+  <dimension ref="A1:AF41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5954,8 +6079,634 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>QFDOS-036</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Benztropina</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Benztropine</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Antagonistas muscarinicos</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Eter tropanico</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>CHEMBL1201203</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>CN1[C@@H]2CC[C@H]1C[C@@H](OC(c1ccccc1)c1ccccc1)C2</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>CN1[C@@H]2CC[C@H]1C[C@@H](OC(c1ccccc1)c1ccccc1)C2</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>CN1[C@@H]2CC[C@H]1C[C@@H](OC(c1ccccc1)c1ccccc1)C2</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>C21H25NO</t>
+        </is>
+      </c>
+      <c r="M37" t="n">
+        <v>307.44</v>
+      </c>
+      <c r="N37" t="n">
+        <v>307.1936</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>93.41</v>
+      </c>
+      <c r="R37" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="S37" t="n">
+        <v>0</v>
+      </c>
+      <c r="T37" t="n">
+        <v>2</v>
+      </c>
+      <c r="U37" t="n">
+        <v>4</v>
+      </c>
+      <c r="V37" t="n">
+        <v>23</v>
+      </c>
+      <c r="W37" t="n">
+        <v>4</v>
+      </c>
+      <c r="X37" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>0.429</v>
+      </c>
+      <c r="Z37" t="n">
+        <v>0.829</v>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>C3:R; C6:S; C8:r</t>
+        </is>
+      </c>
+      <c r="AB37" t="inlineStr">
+        <is>
+          <t>GIJXKZJWITVLHI-PMOLBWCYSA-N</t>
+        </is>
+      </c>
+      <c r="AC37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="AE37" t="inlineStr">
+        <is>
+          <t>img/QFDOS-036_benztropina.png</t>
+        </is>
+      </c>
+      <c r="AF37" t="inlineStr">
+        <is>
+          <t>Hibrido de las dos series del curso: conserva intacto el tropano de la atropina y le acopla el eter de benzhidrilo de la difenhidramina. El cambio funcional decisivo es ester por eter: sin carbonilo no hay hidrolisis por esterasas y desaparecen dos aceptores polares, de modo que la TPSA cae a 12.47, la mas baja de toda la base, con logP 4.42. Amina terciaria mas esa combinacion de polaridad minima y lipofilia alta: entra en SNC con facilidad y se usa como antiparkinsoniano (ATC N04AC01) por bloqueo muscarinico estriatal, igual que el trihexifenidilo, pero ademas inhibe el transportador de dopamina (DAT), un mecanismo dopaminergico adicional que el trihexifenidilo no tiene. Estereoquimica: los dos cabeza de puente del tropano estan definidos y el carbono bencidrilico NO es estereocentro, porque lleva dos fenilos identicos; por eso, a diferencia de la atropina, no hay centro sin definir ni racemato. Se maneja como mesilato (CHEMBL1200383, Cogentin). Verificado contra ChEMBL: CHEMBL1201203, coincidencia exacta de SMILES, InChIKey, MW, logP, TPSA y QED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>QFDOS-037</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Succinilcolina</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Succinylcholine</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Bloqueantes neuromusculares</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Bis-ester de colina</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>C[N+](C)(C)CCOC(=O)CCC(=O)OCC[N+](C)(C)C</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>C[N+](C)(C)CCOC(=O)CCC(=O)OCC[N+](C)(C)C</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>2</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>C[N+](C)(C)CCOC(=O)CCC(=O)OCC[N+](C)(C)C</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>C14H30N2O4+2</t>
+        </is>
+      </c>
+      <c r="M38" t="n">
+        <v>290.4</v>
+      </c>
+      <c r="N38" t="n">
+        <v>290.2195</v>
+      </c>
+      <c r="O38" t="n">
+        <v>2</v>
+      </c>
+      <c r="P38" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>76.95</v>
+      </c>
+      <c r="R38" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="S38" t="n">
+        <v>0</v>
+      </c>
+      <c r="T38" t="n">
+        <v>4</v>
+      </c>
+      <c r="U38" t="n">
+        <v>9</v>
+      </c>
+      <c r="V38" t="n">
+        <v>20</v>
+      </c>
+      <c r="W38" t="n">
+        <v>0</v>
+      </c>
+      <c r="X38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>0.857</v>
+      </c>
+      <c r="Z38" t="n">
+        <v>0.452</v>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>aquiral</t>
+        </is>
+      </c>
+      <c r="AB38" t="inlineStr">
+        <is>
+          <t>AXOIZCJOOAYSMI-UHFFFAOYSA-N</t>
+        </is>
+      </c>
+      <c r="AC38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="AE38" t="inlineStr">
+        <is>
+          <t>img/QFDOS-037_succinilcolina.png</t>
+        </is>
+      </c>
+      <c r="AF38" t="inlineStr">
+        <is>
+          <t>Suxametonio: literalmente dos moleculas de acetilcolina unidas por sus extremos acetilo, es decir el diester de acido succinico con dos colinas. Esa es toda la idea de diseno y se ve de un vistazo junto a QFDOS-001. Bloqueante neuromuscular DESPOLARIZANTE, el unico de la base: en lugar de antagonizar el receptor nicotinico lo activa de forma persistente, porque no lo hidroliza la acetilcolinesterasa; la despolarizacion mantenida inactiva los canales de sodio adyacentes y produce el bloqueo, precedido de las fasciculaciones caracteristicas. Contrasta punto por punto con el atracurio (QFDOS-026), que es no despolarizante y competitivo. Duracion ultracorta porque la hidroliza la butirilcolinesterasa plasmatica: en deficit genetico de esa enzima el bloqueo se prolonga durante horas, que es el ejemplo clasico de farmacogenetica del tema. Dication permanente, aquiral, simetrico. Estructura construida a mano (diester succinico de colina) y comprobada con RDKit: C14H30N2O4 2+, 290.40, InChIKey AXOIZCJOOAYSMI-UHFFFAOYSA-N. Pendiente de contrastar contra ChEMBL, que estaba caido el 2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>QFDOS-038</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Pilocarpina</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Pilocarpine</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Agonistas colinergicos</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Alcaloide imidazolico</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>CHEMBL550</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>CC[C@@H]1C(=O)OC[C@@H]1Cc1cncn1C</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>CC[C@@H]1C(=O)OC[C@@H]1Cc1cncn1C</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>CC[C@@H]1C(=O)OC[C@@H]1Cc1cncn1C</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>C11H16N2O2</t>
+        </is>
+      </c>
+      <c r="M39" t="n">
+        <v>208.26</v>
+      </c>
+      <c r="N39" t="n">
+        <v>208.1212</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>55.14</v>
+      </c>
+      <c r="R39" t="n">
+        <v>44.12</v>
+      </c>
+      <c r="S39" t="n">
+        <v>0</v>
+      </c>
+      <c r="T39" t="n">
+        <v>3</v>
+      </c>
+      <c r="U39" t="n">
+        <v>3</v>
+      </c>
+      <c r="V39" t="n">
+        <v>15</v>
+      </c>
+      <c r="W39" t="n">
+        <v>2</v>
+      </c>
+      <c r="X39" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>0.636</v>
+      </c>
+      <c r="Z39" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>C3:S; C8:R</t>
+        </is>
+      </c>
+      <c r="AB39" t="inlineStr">
+        <is>
+          <t>QCHFTSOMWOSFHM-WPRPVWTQSA-N</t>
+        </is>
+      </c>
+      <c r="AC39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="AE39" t="inlineStr">
+        <is>
+          <t>img/QFDOS-038_pilocarpina.png</t>
+        </is>
+      </c>
+      <c r="AF39" t="inlineStr">
+        <is>
+          <t>El agonista muscarinico que rompe el molde del bloque: ni ester de colina ni amonio cuaternario. Alcaloide de Pilocarpus jaborandi formado por una gamma-butirolactona con un etilo y un metilimidazol. El imidazol basico (pKa en torno a 7) hace el papel del nitrogeno cationico frente al receptor, pero a pH 7.4 una fraccion apreciable esta sin protonar, de modo que atraviesa membranas: por eso es activa por via topica ocular y tambien por via oral, al reves que la muscarina, que es cuaternaria y queda confinada. Ese contraste entre dos agonistas naturales, uno cuaternario y otro base terciaria, es el mejor argumento del tema para separar farmacoforo de propiedades fisicoquimicas. Usos: glaucoma (la miosis tracciona del trabeculo y facilita el drenaje del humor acuoso) y xerostomia en sindrome de Sjogren y tras radioterapia de cabeza y cuello. ATC S01EB01 y N07AX01. Aviso de formulacion: la lactona se hidroliza y epimeriza en medio basico a isopilocarpina, practicamente inactiva, lo que obliga a formular los colirios a pH acido. Estereoquimica cis (3S,4R): los dos sustituyentes del anillo de lactona quedan del mismo lado, y la isopilocarpina es el epimero trans. Verificado contra ChEMBL: CHEMBL550, coincidencia exacta de SMILES, InChIKey, MW, logP, TPSA y QED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>QFDOS-039</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Biperideno</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Biperiden</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Antagonistas muscarinicos</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Aminopropanol</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>CHEMBL1101</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>OC(CCN1CCCCC1)(c1ccccc1)C1CC2C=CC1C2</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>OC(CCN1CCCCC1)(c1ccccc1)C1CC2C=CC1C2</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>OC(CCN1CCCCC1)(c1ccccc1)C1CC2C=CC1C2</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>C21H29NO</t>
+        </is>
+      </c>
+      <c r="M40" t="n">
+        <v>311.47</v>
+      </c>
+      <c r="N40" t="n">
+        <v>311.2249</v>
+      </c>
+      <c r="O40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>94.09</v>
+      </c>
+      <c r="R40" t="n">
+        <v>23.47</v>
+      </c>
+      <c r="S40" t="n">
+        <v>1</v>
+      </c>
+      <c r="T40" t="n">
+        <v>2</v>
+      </c>
+      <c r="U40" t="n">
+        <v>5</v>
+      </c>
+      <c r="V40" t="n">
+        <v>23</v>
+      </c>
+      <c r="W40" t="n">
+        <v>4</v>
+      </c>
+      <c r="X40" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>0.619</v>
+      </c>
+      <c r="Z40" t="n">
+        <v>0.832</v>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>4 centro(s) sin definir</t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>YSXKPIUOCJLQIE-UHFFFAOYSA-N</t>
+        </is>
+      </c>
+      <c r="AC40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="AE40" t="inlineStr">
+        <is>
+          <t>img/QFDOS-039_biperideno.png</t>
+        </is>
+      </c>
+      <c r="AF40" t="inlineStr">
+        <is>
+          <t>Trihexifenidilo con el ciclohexilo sustituido por un biciclo[2.2.1]hept-5-en-2-ilo (norbornenilo). Mismo farmacoforo de aminopropanol: carbinol terciario, fenilo, resto voluminoso saturado y amina ciclica; la piperidina se conserva. El norborneno es mas rigido y mas voluminoso que el ciclohexilo, y baja ligeramente la lipofilia (logP 3.96 frente a 4.33). Antiparkinsoniano y correctors del parkinsonismo inducido por neurolepticos, con presentacion inyectable para la distonia aguda, que es su ventaja practica frente al trihexifenidilo. ATC N04AA02. Estereoquimica: el carbinol y el norborneno generan varios centros que ChEMBL deja sin definir porque se emplea como mezcla; se conserva asi. Verificado contra ChEMBL: CHEMBL1101, coincidencia exacta de SMILES, InChIKey, MW, logP, TPSA y QED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>QFDOS-040</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Prociclidina</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Procyclidine</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Antagonistas muscarinicos</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Aminopropanol</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>CHEMBL86715</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>OC(CCN1CCCC1)(c1ccccc1)C1CCCCC1</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>OC(CCN1CCCC1)(c1ccccc1)C1CCCCC1</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>OC(CCN1CCCC1)(c1ccccc1)C1CCCCC1</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>C19H29NO</t>
+        </is>
+      </c>
+      <c r="M41" t="n">
+        <v>287.45</v>
+      </c>
+      <c r="N41" t="n">
+        <v>287.2249</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="R41" t="n">
+        <v>23.47</v>
+      </c>
+      <c r="S41" t="n">
+        <v>1</v>
+      </c>
+      <c r="T41" t="n">
+        <v>2</v>
+      </c>
+      <c r="U41" t="n">
+        <v>5</v>
+      </c>
+      <c r="V41" t="n">
+        <v>21</v>
+      </c>
+      <c r="W41" t="n">
+        <v>3</v>
+      </c>
+      <c r="X41" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>0.6840000000000001</v>
+      </c>
+      <c r="Z41" t="n">
+        <v>0.886</v>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>1 centro(s) sin definir</t>
+        </is>
+      </c>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>WYDUSKDSKCASEF-UHFFFAOYSA-N</t>
+        </is>
+      </c>
+      <c r="AC41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="AE41" t="inlineStr">
+        <is>
+          <t>img/QFDOS-040_prociclidina.png</t>
+        </is>
+      </c>
+      <c r="AF41" t="inlineStr">
+        <is>
+          <t>Trihexifenidilo con pirrolidina en lugar de piperidina: un solo carbono menos en el anillo de la amina basica, sin tocar nada mas. Es la variacion mas pequena de toda la base y sirve para preguntar en clase que cambia y que no: la firma polar es identica (TPSA 23.47) y la lipofilia practicamente tambien (logP 3.94 frente a 4.33), de modo que el efecto del cambio hay que buscarlo en la geometria del nitrogeno, no en los descriptores globales. Antiparkinsoniano y correctors del parkinsonismo por neurolepticos. ATC N04AA04. El sufijo -clidine de la DCI marca agonistas y antagonistas muscarinicos. Estereoquimica: el carbinol es estereocentro y ChEMBL lo deja sin definir (se emplea como racemico); se conserva asi. Verificado contra ChEMBL: CHEMBL86715, coincidencia exacta de SMILES, InChIKey, MW, logP, TPSA y QED.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AF36"/>
+  <autoFilter ref="A1:AF41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5966,7 +6717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6592,6 +7343,91 @@
         </is>
       </c>
     </row>
+    <row r="37" ht="155" customHeight="1">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>QFDOS-036</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Benztropina</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>C21H25NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="155" customHeight="1">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>QFDOS-037</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Succinilcolina</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>C14H30N2O4+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="155" customHeight="1">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>QFDOS-038</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Pilocarpina</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>C11H16N2O2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="155" customHeight="1">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>QFDOS-039</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Biperideno</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>C21H29NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="155" customHeight="1">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>QFDOS-040</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Prociclidina</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>C19H29NO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>